<commit_message>
NEW: Código manual terminado
</commit_message>
<xml_diff>
--- a/resultados_globales.xlsx
+++ b/resultados_globales.xlsx
@@ -5,17 +5,18 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\juanp\Documents\Semestre VII\Paralela\codigo\proyecto_parcial2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\juanp\Desktop\GIT\parcial_2_paralela\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C8B9707-9419-4153-9A02-BB69B139090D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEC2F6A7-81BF-41C8-8F05-8132F5D41227}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="resultados_secuencial" sheetId="5" r:id="rId1"/>
     <sheet name="resultados_paralelo_ia" sheetId="6" r:id="rId2"/>
     <sheet name="resultados_paralelo_ia_opt" sheetId="7" r:id="rId3"/>
+    <sheet name="resultados_paralelo_manual" sheetId="8" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="15">
   <si>
     <t>Variante</t>
   </si>
@@ -81,6 +82,9 @@
   <si>
     <t>Paralelo_IA_Opt</t>
   </si>
+  <si>
+    <t>Paralelo_Manual</t>
+  </si>
 </sst>
 </file>
 
@@ -115,8 +119,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6705,4 +6710,2850 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDA1813F-8E51-4234-9F7C-9CCF234C42C1}">
+  <dimension ref="A1:M81"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2">
+        <v>512</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>30</v>
+      </c>
+      <c r="F2">
+        <v>3.3035999999999999</v>
+      </c>
+      <c r="G2">
+        <v>0.41260000000000002</v>
+      </c>
+      <c r="H2">
+        <v>2.8266</v>
+      </c>
+      <c r="I2">
+        <v>4.9980000000000002</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3">
+        <v>512</v>
+      </c>
+      <c r="C3">
+        <v>3</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3">
+        <v>30</v>
+      </c>
+      <c r="F3">
+        <v>2.2370000000000001</v>
+      </c>
+      <c r="G3">
+        <v>0.2802</v>
+      </c>
+      <c r="H3">
+        <v>1.8677999999999999</v>
+      </c>
+      <c r="I3">
+        <v>3.2267000000000001</v>
+      </c>
+      <c r="J3">
+        <v>1.4767999999999999</v>
+      </c>
+      <c r="K3">
+        <v>0.73839999999999995</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4">
+        <v>512</v>
+      </c>
+      <c r="C4">
+        <v>3</v>
+      </c>
+      <c r="D4">
+        <v>4</v>
+      </c>
+      <c r="E4">
+        <v>30</v>
+      </c>
+      <c r="F4">
+        <v>1.7010000000000001</v>
+      </c>
+      <c r="G4">
+        <v>0.25640000000000002</v>
+      </c>
+      <c r="H4">
+        <v>1.3424</v>
+      </c>
+      <c r="I4">
+        <v>2.5003000000000002</v>
+      </c>
+      <c r="J4">
+        <v>1.9420999999999999</v>
+      </c>
+      <c r="K4">
+        <v>0.48549999999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5">
+        <v>512</v>
+      </c>
+      <c r="C5">
+        <v>3</v>
+      </c>
+      <c r="D5">
+        <v>8</v>
+      </c>
+      <c r="E5">
+        <v>30</v>
+      </c>
+      <c r="F5">
+        <v>1.8219000000000001</v>
+      </c>
+      <c r="G5">
+        <v>0.45739999999999997</v>
+      </c>
+      <c r="H5">
+        <v>1.1773</v>
+      </c>
+      <c r="I5">
+        <v>2.9979</v>
+      </c>
+      <c r="J5">
+        <v>1.8131999999999999</v>
+      </c>
+      <c r="K5">
+        <v>0.22670000000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6">
+        <v>512</v>
+      </c>
+      <c r="C6">
+        <v>3</v>
+      </c>
+      <c r="D6">
+        <v>16</v>
+      </c>
+      <c r="E6">
+        <v>30</v>
+      </c>
+      <c r="F6">
+        <v>2.1528999999999998</v>
+      </c>
+      <c r="G6">
+        <v>0.47539999999999999</v>
+      </c>
+      <c r="H6">
+        <v>1.5007999999999999</v>
+      </c>
+      <c r="I6">
+        <v>3.2770999999999999</v>
+      </c>
+      <c r="J6">
+        <v>1.5345</v>
+      </c>
+      <c r="K6">
+        <v>9.5899999999999999E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7">
+        <v>512</v>
+      </c>
+      <c r="C7">
+        <v>5</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>30</v>
+      </c>
+      <c r="F7">
+        <v>6.0613999999999999</v>
+      </c>
+      <c r="G7">
+        <v>0.39829999999999999</v>
+      </c>
+      <c r="H7">
+        <v>5.4378000000000002</v>
+      </c>
+      <c r="I7">
+        <v>7.0083000000000002</v>
+      </c>
+      <c r="J7">
+        <v>1</v>
+      </c>
+      <c r="K7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8">
+        <v>512</v>
+      </c>
+      <c r="C8">
+        <v>5</v>
+      </c>
+      <c r="D8">
+        <v>2</v>
+      </c>
+      <c r="E8">
+        <v>30</v>
+      </c>
+      <c r="F8">
+        <v>4.1199000000000003</v>
+      </c>
+      <c r="G8">
+        <v>0.68430000000000002</v>
+      </c>
+      <c r="H8">
+        <v>3.3443000000000001</v>
+      </c>
+      <c r="I8">
+        <v>6.3555999999999999</v>
+      </c>
+      <c r="J8">
+        <v>1.4712000000000001</v>
+      </c>
+      <c r="K8">
+        <v>0.73560000000000003</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9">
+        <v>512</v>
+      </c>
+      <c r="C9">
+        <v>5</v>
+      </c>
+      <c r="D9">
+        <v>4</v>
+      </c>
+      <c r="E9">
+        <v>30</v>
+      </c>
+      <c r="F9">
+        <v>2.8203</v>
+      </c>
+      <c r="G9">
+        <v>0.49249999999999999</v>
+      </c>
+      <c r="H9">
+        <v>2.1333000000000002</v>
+      </c>
+      <c r="I9">
+        <v>4.1346999999999996</v>
+      </c>
+      <c r="J9">
+        <v>2.1492</v>
+      </c>
+      <c r="K9">
+        <v>0.5373</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10">
+        <v>512</v>
+      </c>
+      <c r="C10">
+        <v>5</v>
+      </c>
+      <c r="D10">
+        <v>8</v>
+      </c>
+      <c r="E10">
+        <v>30</v>
+      </c>
+      <c r="F10">
+        <v>2.1465000000000001</v>
+      </c>
+      <c r="G10">
+        <v>0.51780000000000004</v>
+      </c>
+      <c r="H10">
+        <v>1.4831000000000001</v>
+      </c>
+      <c r="I10">
+        <v>3.9239999999999999</v>
+      </c>
+      <c r="J10">
+        <v>2.8239000000000001</v>
+      </c>
+      <c r="K10">
+        <v>0.35299999999999998</v>
+      </c>
+      <c r="M10" s="1"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11">
+        <v>512</v>
+      </c>
+      <c r="C11">
+        <v>5</v>
+      </c>
+      <c r="D11">
+        <v>16</v>
+      </c>
+      <c r="E11">
+        <v>30</v>
+      </c>
+      <c r="F11">
+        <v>1.982</v>
+      </c>
+      <c r="G11">
+        <v>0.23400000000000001</v>
+      </c>
+      <c r="H11">
+        <v>1.7338</v>
+      </c>
+      <c r="I11">
+        <v>2.7071000000000001</v>
+      </c>
+      <c r="J11">
+        <v>3.0581999999999998</v>
+      </c>
+      <c r="K11">
+        <v>0.19109999999999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12">
+        <v>512</v>
+      </c>
+      <c r="C12">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12">
+        <v>30</v>
+      </c>
+      <c r="F12">
+        <v>10.1745</v>
+      </c>
+      <c r="G12">
+        <v>0.22359999999999999</v>
+      </c>
+      <c r="H12">
+        <v>9.8519000000000005</v>
+      </c>
+      <c r="I12">
+        <v>10.9564</v>
+      </c>
+      <c r="J12">
+        <v>1</v>
+      </c>
+      <c r="K12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13">
+        <v>512</v>
+      </c>
+      <c r="C13">
+        <v>7</v>
+      </c>
+      <c r="D13">
+        <v>2</v>
+      </c>
+      <c r="E13">
+        <v>30</v>
+      </c>
+      <c r="F13">
+        <v>5.6130000000000004</v>
+      </c>
+      <c r="G13">
+        <v>0.30580000000000002</v>
+      </c>
+      <c r="H13">
+        <v>5.3436000000000003</v>
+      </c>
+      <c r="I13">
+        <v>6.9756</v>
+      </c>
+      <c r="J13">
+        <v>1.8126</v>
+      </c>
+      <c r="K13">
+        <v>0.90629999999999999</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14">
+        <v>512</v>
+      </c>
+      <c r="C14">
+        <v>7</v>
+      </c>
+      <c r="D14">
+        <v>4</v>
+      </c>
+      <c r="E14">
+        <v>30</v>
+      </c>
+      <c r="F14">
+        <v>3.391</v>
+      </c>
+      <c r="G14">
+        <v>0.26519999999999999</v>
+      </c>
+      <c r="H14">
+        <v>3.1091000000000002</v>
+      </c>
+      <c r="I14">
+        <v>4.5538999999999996</v>
+      </c>
+      <c r="J14">
+        <v>3.0004</v>
+      </c>
+      <c r="K14">
+        <v>0.75009999999999999</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15">
+        <v>512</v>
+      </c>
+      <c r="C15">
+        <v>7</v>
+      </c>
+      <c r="D15">
+        <v>8</v>
+      </c>
+      <c r="E15">
+        <v>30</v>
+      </c>
+      <c r="F15">
+        <v>2.6993999999999998</v>
+      </c>
+      <c r="G15">
+        <v>0.47889999999999999</v>
+      </c>
+      <c r="H15">
+        <v>2.1392000000000002</v>
+      </c>
+      <c r="I15">
+        <v>4.1257999999999999</v>
+      </c>
+      <c r="J15">
+        <v>3.7692000000000001</v>
+      </c>
+      <c r="K15">
+        <v>0.47120000000000001</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16">
+        <v>512</v>
+      </c>
+      <c r="C16">
+        <v>7</v>
+      </c>
+      <c r="D16">
+        <v>16</v>
+      </c>
+      <c r="E16">
+        <v>30</v>
+      </c>
+      <c r="F16">
+        <v>2.6278999999999999</v>
+      </c>
+      <c r="G16">
+        <v>0.34720000000000001</v>
+      </c>
+      <c r="H16">
+        <v>2.1137000000000001</v>
+      </c>
+      <c r="I16">
+        <v>3.3631000000000002</v>
+      </c>
+      <c r="J16">
+        <v>3.8717999999999999</v>
+      </c>
+      <c r="K16">
+        <v>0.24199999999999999</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17">
+        <v>512</v>
+      </c>
+      <c r="C17">
+        <v>11</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17">
+        <v>30</v>
+      </c>
+      <c r="F17">
+        <v>25.687200000000001</v>
+      </c>
+      <c r="G17">
+        <v>0.50700000000000001</v>
+      </c>
+      <c r="H17">
+        <v>24.816800000000001</v>
+      </c>
+      <c r="I17">
+        <v>27.449000000000002</v>
+      </c>
+      <c r="J17">
+        <v>1</v>
+      </c>
+      <c r="K17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>14</v>
+      </c>
+      <c r="B18">
+        <v>512</v>
+      </c>
+      <c r="C18">
+        <v>11</v>
+      </c>
+      <c r="D18">
+        <v>2</v>
+      </c>
+      <c r="E18">
+        <v>30</v>
+      </c>
+      <c r="F18">
+        <v>13.4239</v>
+      </c>
+      <c r="G18">
+        <v>0.2087</v>
+      </c>
+      <c r="H18">
+        <v>13.136100000000001</v>
+      </c>
+      <c r="I18">
+        <v>14.0428</v>
+      </c>
+      <c r="J18">
+        <v>1.9135</v>
+      </c>
+      <c r="K18">
+        <v>0.95679999999999998</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>14</v>
+      </c>
+      <c r="B19">
+        <v>512</v>
+      </c>
+      <c r="C19">
+        <v>11</v>
+      </c>
+      <c r="D19">
+        <v>4</v>
+      </c>
+      <c r="E19">
+        <v>30</v>
+      </c>
+      <c r="F19">
+        <v>7.3761000000000001</v>
+      </c>
+      <c r="G19">
+        <v>0.52780000000000005</v>
+      </c>
+      <c r="H19">
+        <v>6.9038000000000004</v>
+      </c>
+      <c r="I19">
+        <v>9.0881000000000007</v>
+      </c>
+      <c r="J19">
+        <v>3.4824999999999999</v>
+      </c>
+      <c r="K19">
+        <v>0.87060000000000004</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>14</v>
+      </c>
+      <c r="B20">
+        <v>512</v>
+      </c>
+      <c r="C20">
+        <v>11</v>
+      </c>
+      <c r="D20">
+        <v>8</v>
+      </c>
+      <c r="E20">
+        <v>30</v>
+      </c>
+      <c r="F20">
+        <v>5.298</v>
+      </c>
+      <c r="G20">
+        <v>0.93310000000000004</v>
+      </c>
+      <c r="H20">
+        <v>4.0914999999999999</v>
+      </c>
+      <c r="I20">
+        <v>6.9085999999999999</v>
+      </c>
+      <c r="J20">
+        <v>4.8483999999999998</v>
+      </c>
+      <c r="K20">
+        <v>0.60609999999999997</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>14</v>
+      </c>
+      <c r="B21">
+        <v>512</v>
+      </c>
+      <c r="C21">
+        <v>11</v>
+      </c>
+      <c r="D21">
+        <v>16</v>
+      </c>
+      <c r="E21">
+        <v>30</v>
+      </c>
+      <c r="F21">
+        <v>4.4626999999999999</v>
+      </c>
+      <c r="G21">
+        <v>0.5252</v>
+      </c>
+      <c r="H21">
+        <v>3.6917</v>
+      </c>
+      <c r="I21">
+        <v>5.5621</v>
+      </c>
+      <c r="J21">
+        <v>5.7560000000000002</v>
+      </c>
+      <c r="K21">
+        <v>0.35970000000000002</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>14</v>
+      </c>
+      <c r="B22">
+        <v>1024</v>
+      </c>
+      <c r="C22">
+        <v>3</v>
+      </c>
+      <c r="D22">
+        <v>1</v>
+      </c>
+      <c r="E22">
+        <v>30</v>
+      </c>
+      <c r="F22">
+        <v>9.8088999999999995</v>
+      </c>
+      <c r="G22">
+        <v>0.2288</v>
+      </c>
+      <c r="H22">
+        <v>9.4977</v>
+      </c>
+      <c r="I22">
+        <v>10.298999999999999</v>
+      </c>
+      <c r="J22">
+        <v>1</v>
+      </c>
+      <c r="K22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>14</v>
+      </c>
+      <c r="B23">
+        <v>1024</v>
+      </c>
+      <c r="C23">
+        <v>3</v>
+      </c>
+      <c r="D23">
+        <v>2</v>
+      </c>
+      <c r="E23">
+        <v>30</v>
+      </c>
+      <c r="F23">
+        <v>5.5096999999999996</v>
+      </c>
+      <c r="G23">
+        <v>0.28710000000000002</v>
+      </c>
+      <c r="H23">
+        <v>5.0963000000000003</v>
+      </c>
+      <c r="I23">
+        <v>6.5247999999999999</v>
+      </c>
+      <c r="J23">
+        <v>1.7803</v>
+      </c>
+      <c r="K23">
+        <v>0.89019999999999999</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>14</v>
+      </c>
+      <c r="B24">
+        <v>1024</v>
+      </c>
+      <c r="C24">
+        <v>3</v>
+      </c>
+      <c r="D24">
+        <v>4</v>
+      </c>
+      <c r="E24">
+        <v>30</v>
+      </c>
+      <c r="F24">
+        <v>3.3847999999999998</v>
+      </c>
+      <c r="G24">
+        <v>0.2853</v>
+      </c>
+      <c r="H24">
+        <v>3.0657999999999999</v>
+      </c>
+      <c r="I24">
+        <v>4.4793000000000003</v>
+      </c>
+      <c r="J24">
+        <v>2.8978999999999999</v>
+      </c>
+      <c r="K24">
+        <v>0.72450000000000003</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>14</v>
+      </c>
+      <c r="B25">
+        <v>1024</v>
+      </c>
+      <c r="C25">
+        <v>3</v>
+      </c>
+      <c r="D25">
+        <v>8</v>
+      </c>
+      <c r="E25">
+        <v>30</v>
+      </c>
+      <c r="F25">
+        <v>2.8694999999999999</v>
+      </c>
+      <c r="G25">
+        <v>0.49159999999999998</v>
+      </c>
+      <c r="H25">
+        <v>2.1410999999999998</v>
+      </c>
+      <c r="I25">
+        <v>3.6718999999999999</v>
+      </c>
+      <c r="J25">
+        <v>3.4182999999999999</v>
+      </c>
+      <c r="K25">
+        <v>0.42730000000000001</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>14</v>
+      </c>
+      <c r="B26">
+        <v>1024</v>
+      </c>
+      <c r="C26">
+        <v>3</v>
+      </c>
+      <c r="D26">
+        <v>16</v>
+      </c>
+      <c r="E26">
+        <v>30</v>
+      </c>
+      <c r="F26">
+        <v>2.7029999999999998</v>
+      </c>
+      <c r="G26">
+        <v>0.4763</v>
+      </c>
+      <c r="H26">
+        <v>2.3275000000000001</v>
+      </c>
+      <c r="I26">
+        <v>4.2321999999999997</v>
+      </c>
+      <c r="J26">
+        <v>3.6288</v>
+      </c>
+      <c r="K26">
+        <v>0.2268</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>14</v>
+      </c>
+      <c r="B27">
+        <v>1024</v>
+      </c>
+      <c r="C27">
+        <v>5</v>
+      </c>
+      <c r="D27">
+        <v>1</v>
+      </c>
+      <c r="E27">
+        <v>30</v>
+      </c>
+      <c r="F27">
+        <v>20.8718</v>
+      </c>
+      <c r="G27">
+        <v>0.21540000000000001</v>
+      </c>
+      <c r="H27">
+        <v>20.310199999999998</v>
+      </c>
+      <c r="I27">
+        <v>21.443200000000001</v>
+      </c>
+      <c r="J27">
+        <v>1</v>
+      </c>
+      <c r="K27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>14</v>
+      </c>
+      <c r="B28">
+        <v>1024</v>
+      </c>
+      <c r="C28">
+        <v>5</v>
+      </c>
+      <c r="D28">
+        <v>2</v>
+      </c>
+      <c r="E28">
+        <v>30</v>
+      </c>
+      <c r="F28">
+        <v>11.169499999999999</v>
+      </c>
+      <c r="G28">
+        <v>0.53300000000000003</v>
+      </c>
+      <c r="H28">
+        <v>10.733700000000001</v>
+      </c>
+      <c r="I28">
+        <v>13.2264</v>
+      </c>
+      <c r="J28">
+        <v>1.8686</v>
+      </c>
+      <c r="K28">
+        <v>0.93430000000000002</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>14</v>
+      </c>
+      <c r="B29">
+        <v>1024</v>
+      </c>
+      <c r="C29">
+        <v>5</v>
+      </c>
+      <c r="D29">
+        <v>4</v>
+      </c>
+      <c r="E29">
+        <v>30</v>
+      </c>
+      <c r="F29">
+        <v>6.3723999999999998</v>
+      </c>
+      <c r="G29">
+        <v>0.55279999999999996</v>
+      </c>
+      <c r="H29">
+        <v>5.8071999999999999</v>
+      </c>
+      <c r="I29">
+        <v>8.0556999999999999</v>
+      </c>
+      <c r="J29">
+        <v>3.2753999999999999</v>
+      </c>
+      <c r="K29">
+        <v>0.81879999999999997</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>14</v>
+      </c>
+      <c r="B30">
+        <v>1024</v>
+      </c>
+      <c r="C30">
+        <v>5</v>
+      </c>
+      <c r="D30">
+        <v>8</v>
+      </c>
+      <c r="E30">
+        <v>30</v>
+      </c>
+      <c r="F30">
+        <v>4.8413000000000004</v>
+      </c>
+      <c r="G30">
+        <v>1.0133000000000001</v>
+      </c>
+      <c r="H30">
+        <v>3.5781000000000001</v>
+      </c>
+      <c r="I30">
+        <v>6.5486000000000004</v>
+      </c>
+      <c r="J30">
+        <v>4.3112000000000004</v>
+      </c>
+      <c r="K30">
+        <v>0.53890000000000005</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>14</v>
+      </c>
+      <c r="B31">
+        <v>1024</v>
+      </c>
+      <c r="C31">
+        <v>5</v>
+      </c>
+      <c r="D31">
+        <v>16</v>
+      </c>
+      <c r="E31">
+        <v>30</v>
+      </c>
+      <c r="F31">
+        <v>4.6017000000000001</v>
+      </c>
+      <c r="G31">
+        <v>0.59360000000000002</v>
+      </c>
+      <c r="H31">
+        <v>3.6455000000000002</v>
+      </c>
+      <c r="I31">
+        <v>5.8533999999999997</v>
+      </c>
+      <c r="J31">
+        <v>4.5357000000000003</v>
+      </c>
+      <c r="K31">
+        <v>0.28349999999999997</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>14</v>
+      </c>
+      <c r="B32">
+        <v>1024</v>
+      </c>
+      <c r="C32">
+        <v>7</v>
+      </c>
+      <c r="D32">
+        <v>1</v>
+      </c>
+      <c r="E32">
+        <v>30</v>
+      </c>
+      <c r="F32">
+        <v>38.907800000000002</v>
+      </c>
+      <c r="G32">
+        <v>0.58299999999999996</v>
+      </c>
+      <c r="H32">
+        <v>38.1982</v>
+      </c>
+      <c r="I32">
+        <v>40.361600000000003</v>
+      </c>
+      <c r="J32">
+        <v>1</v>
+      </c>
+      <c r="K32">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>14</v>
+      </c>
+      <c r="B33">
+        <v>1024</v>
+      </c>
+      <c r="C33">
+        <v>7</v>
+      </c>
+      <c r="D33">
+        <v>2</v>
+      </c>
+      <c r="E33">
+        <v>30</v>
+      </c>
+      <c r="F33">
+        <v>20.1584</v>
+      </c>
+      <c r="G33">
+        <v>0.43559999999999999</v>
+      </c>
+      <c r="H33">
+        <v>19.6935</v>
+      </c>
+      <c r="I33">
+        <v>22.038499999999999</v>
+      </c>
+      <c r="J33">
+        <v>1.9300999999999999</v>
+      </c>
+      <c r="K33">
+        <v>0.96509999999999996</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>14</v>
+      </c>
+      <c r="B34">
+        <v>1024</v>
+      </c>
+      <c r="C34">
+        <v>7</v>
+      </c>
+      <c r="D34">
+        <v>4</v>
+      </c>
+      <c r="E34">
+        <v>30</v>
+      </c>
+      <c r="F34">
+        <v>11.1089</v>
+      </c>
+      <c r="G34">
+        <v>0.90049999999999997</v>
+      </c>
+      <c r="H34">
+        <v>10.3545</v>
+      </c>
+      <c r="I34">
+        <v>14.485099999999999</v>
+      </c>
+      <c r="J34">
+        <v>3.5024000000000002</v>
+      </c>
+      <c r="K34">
+        <v>0.87560000000000004</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>14</v>
+      </c>
+      <c r="B35">
+        <v>1024</v>
+      </c>
+      <c r="C35">
+        <v>7</v>
+      </c>
+      <c r="D35">
+        <v>8</v>
+      </c>
+      <c r="E35">
+        <v>30</v>
+      </c>
+      <c r="F35">
+        <v>7.5772000000000004</v>
+      </c>
+      <c r="G35">
+        <v>1.2803</v>
+      </c>
+      <c r="H35">
+        <v>5.8876999999999997</v>
+      </c>
+      <c r="I35">
+        <v>10.401300000000001</v>
+      </c>
+      <c r="J35">
+        <v>5.1348000000000003</v>
+      </c>
+      <c r="K35">
+        <v>0.64190000000000003</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>14</v>
+      </c>
+      <c r="B36">
+        <v>1024</v>
+      </c>
+      <c r="C36">
+        <v>7</v>
+      </c>
+      <c r="D36">
+        <v>16</v>
+      </c>
+      <c r="E36">
+        <v>30</v>
+      </c>
+      <c r="F36">
+        <v>6.6829999999999998</v>
+      </c>
+      <c r="G36">
+        <v>1.0024999999999999</v>
+      </c>
+      <c r="H36">
+        <v>5.5077999999999996</v>
+      </c>
+      <c r="I36">
+        <v>8.7411999999999992</v>
+      </c>
+      <c r="J36">
+        <v>5.8219000000000003</v>
+      </c>
+      <c r="K36">
+        <v>0.3639</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>14</v>
+      </c>
+      <c r="B37">
+        <v>1024</v>
+      </c>
+      <c r="C37">
+        <v>11</v>
+      </c>
+      <c r="D37">
+        <v>1</v>
+      </c>
+      <c r="E37">
+        <v>30</v>
+      </c>
+      <c r="F37">
+        <v>101.2948</v>
+      </c>
+      <c r="G37">
+        <v>3.8957000000000002</v>
+      </c>
+      <c r="H37">
+        <v>98.866200000000006</v>
+      </c>
+      <c r="I37">
+        <v>118.756</v>
+      </c>
+      <c r="J37">
+        <v>1</v>
+      </c>
+      <c r="K37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>14</v>
+      </c>
+      <c r="B38">
+        <v>1024</v>
+      </c>
+      <c r="C38">
+        <v>11</v>
+      </c>
+      <c r="D38">
+        <v>2</v>
+      </c>
+      <c r="E38">
+        <v>30</v>
+      </c>
+      <c r="F38">
+        <v>52.146000000000001</v>
+      </c>
+      <c r="G38">
+        <v>1.6802999999999999</v>
+      </c>
+      <c r="H38">
+        <v>50.178199999999997</v>
+      </c>
+      <c r="I38">
+        <v>57.054299999999998</v>
+      </c>
+      <c r="J38">
+        <v>1.9424999999999999</v>
+      </c>
+      <c r="K38">
+        <v>0.97130000000000005</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>14</v>
+      </c>
+      <c r="B39">
+        <v>1024</v>
+      </c>
+      <c r="C39">
+        <v>11</v>
+      </c>
+      <c r="D39">
+        <v>4</v>
+      </c>
+      <c r="E39">
+        <v>30</v>
+      </c>
+      <c r="F39">
+        <v>29.4148</v>
+      </c>
+      <c r="G39">
+        <v>3.7359</v>
+      </c>
+      <c r="H39">
+        <v>26.058399999999999</v>
+      </c>
+      <c r="I39">
+        <v>39.408099999999997</v>
+      </c>
+      <c r="J39">
+        <v>3.4437000000000002</v>
+      </c>
+      <c r="K39">
+        <v>0.8609</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>14</v>
+      </c>
+      <c r="B40">
+        <v>1024</v>
+      </c>
+      <c r="C40">
+        <v>11</v>
+      </c>
+      <c r="D40">
+        <v>8</v>
+      </c>
+      <c r="E40">
+        <v>30</v>
+      </c>
+      <c r="F40">
+        <v>18.899000000000001</v>
+      </c>
+      <c r="G40">
+        <v>2.4333999999999998</v>
+      </c>
+      <c r="H40">
+        <v>13.8489</v>
+      </c>
+      <c r="I40">
+        <v>21.996300000000002</v>
+      </c>
+      <c r="J40">
+        <v>5.3597999999999999</v>
+      </c>
+      <c r="K40">
+        <v>0.67</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>14</v>
+      </c>
+      <c r="B41">
+        <v>1024</v>
+      </c>
+      <c r="C41">
+        <v>11</v>
+      </c>
+      <c r="D41">
+        <v>16</v>
+      </c>
+      <c r="E41">
+        <v>30</v>
+      </c>
+      <c r="F41">
+        <v>13.537699999999999</v>
+      </c>
+      <c r="G41">
+        <v>1.4610000000000001</v>
+      </c>
+      <c r="H41">
+        <v>11.624599999999999</v>
+      </c>
+      <c r="I41">
+        <v>16.2624</v>
+      </c>
+      <c r="J41">
+        <v>7.4824000000000002</v>
+      </c>
+      <c r="K41">
+        <v>0.4677</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>14</v>
+      </c>
+      <c r="B42">
+        <v>2048</v>
+      </c>
+      <c r="C42">
+        <v>3</v>
+      </c>
+      <c r="D42">
+        <v>1</v>
+      </c>
+      <c r="E42">
+        <v>30</v>
+      </c>
+      <c r="F42">
+        <v>37.9054</v>
+      </c>
+      <c r="G42">
+        <v>1.1626000000000001</v>
+      </c>
+      <c r="H42">
+        <v>36.531500000000001</v>
+      </c>
+      <c r="I42">
+        <v>42.752200000000002</v>
+      </c>
+      <c r="J42">
+        <v>1</v>
+      </c>
+      <c r="K42">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>14</v>
+      </c>
+      <c r="B43">
+        <v>2048</v>
+      </c>
+      <c r="C43">
+        <v>3</v>
+      </c>
+      <c r="D43">
+        <v>2</v>
+      </c>
+      <c r="E43">
+        <v>30</v>
+      </c>
+      <c r="F43">
+        <v>19.655999999999999</v>
+      </c>
+      <c r="G43">
+        <v>0.7056</v>
+      </c>
+      <c r="H43">
+        <v>18.989100000000001</v>
+      </c>
+      <c r="I43">
+        <v>22.127600000000001</v>
+      </c>
+      <c r="J43">
+        <v>1.9283999999999999</v>
+      </c>
+      <c r="K43">
+        <v>0.96419999999999995</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>14</v>
+      </c>
+      <c r="B44">
+        <v>2048</v>
+      </c>
+      <c r="C44">
+        <v>3</v>
+      </c>
+      <c r="D44">
+        <v>4</v>
+      </c>
+      <c r="E44">
+        <v>30</v>
+      </c>
+      <c r="F44">
+        <v>11.4979</v>
+      </c>
+      <c r="G44">
+        <v>1.8091999999999999</v>
+      </c>
+      <c r="H44">
+        <v>10.1747</v>
+      </c>
+      <c r="I44">
+        <v>17.053999999999998</v>
+      </c>
+      <c r="J44">
+        <v>3.2967</v>
+      </c>
+      <c r="K44">
+        <v>0.82420000000000004</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>14</v>
+      </c>
+      <c r="B45">
+        <v>2048</v>
+      </c>
+      <c r="C45">
+        <v>3</v>
+      </c>
+      <c r="D45">
+        <v>8</v>
+      </c>
+      <c r="E45">
+        <v>30</v>
+      </c>
+      <c r="F45">
+        <v>8.0885999999999996</v>
+      </c>
+      <c r="G45">
+        <v>1.8411</v>
+      </c>
+      <c r="H45">
+        <v>5.8803000000000001</v>
+      </c>
+      <c r="I45">
+        <v>11.401</v>
+      </c>
+      <c r="J45">
+        <v>4.6863000000000001</v>
+      </c>
+      <c r="K45">
+        <v>0.58579999999999999</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>14</v>
+      </c>
+      <c r="B46">
+        <v>2048</v>
+      </c>
+      <c r="C46">
+        <v>3</v>
+      </c>
+      <c r="D46">
+        <v>16</v>
+      </c>
+      <c r="E46">
+        <v>30</v>
+      </c>
+      <c r="F46">
+        <v>7.0884</v>
+      </c>
+      <c r="G46">
+        <v>1.073</v>
+      </c>
+      <c r="H46">
+        <v>5.9619999999999997</v>
+      </c>
+      <c r="I46">
+        <v>9.6852999999999998</v>
+      </c>
+      <c r="J46">
+        <v>5.3475999999999999</v>
+      </c>
+      <c r="K46">
+        <v>0.3342</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>14</v>
+      </c>
+      <c r="B47">
+        <v>2048</v>
+      </c>
+      <c r="C47">
+        <v>5</v>
+      </c>
+      <c r="D47">
+        <v>1</v>
+      </c>
+      <c r="E47">
+        <v>30</v>
+      </c>
+      <c r="F47">
+        <v>81.191500000000005</v>
+      </c>
+      <c r="G47">
+        <v>0.87009999999999998</v>
+      </c>
+      <c r="H47">
+        <v>80.1691</v>
+      </c>
+      <c r="I47">
+        <v>83.283000000000001</v>
+      </c>
+      <c r="J47">
+        <v>1</v>
+      </c>
+      <c r="K47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>14</v>
+      </c>
+      <c r="B48">
+        <v>2048</v>
+      </c>
+      <c r="C48">
+        <v>5</v>
+      </c>
+      <c r="D48">
+        <v>2</v>
+      </c>
+      <c r="E48">
+        <v>30</v>
+      </c>
+      <c r="F48">
+        <v>45.173999999999999</v>
+      </c>
+      <c r="G48">
+        <v>8.8041</v>
+      </c>
+      <c r="H48">
+        <v>40.979700000000001</v>
+      </c>
+      <c r="I48">
+        <v>84.468400000000003</v>
+      </c>
+      <c r="J48">
+        <v>1.7972999999999999</v>
+      </c>
+      <c r="K48">
+        <v>0.89870000000000005</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>14</v>
+      </c>
+      <c r="B49">
+        <v>2048</v>
+      </c>
+      <c r="C49">
+        <v>5</v>
+      </c>
+      <c r="D49">
+        <v>4</v>
+      </c>
+      <c r="E49">
+        <v>30</v>
+      </c>
+      <c r="F49">
+        <v>24.9635</v>
+      </c>
+      <c r="G49">
+        <v>4.3728999999999996</v>
+      </c>
+      <c r="H49">
+        <v>21.387</v>
+      </c>
+      <c r="I49">
+        <v>36.808599999999998</v>
+      </c>
+      <c r="J49">
+        <v>3.2524000000000002</v>
+      </c>
+      <c r="K49">
+        <v>0.81310000000000004</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>14</v>
+      </c>
+      <c r="B50">
+        <v>2048</v>
+      </c>
+      <c r="C50">
+        <v>5</v>
+      </c>
+      <c r="D50">
+        <v>8</v>
+      </c>
+      <c r="E50">
+        <v>30</v>
+      </c>
+      <c r="F50">
+        <v>17.3599</v>
+      </c>
+      <c r="G50">
+        <v>3.4718</v>
+      </c>
+      <c r="H50">
+        <v>11.636699999999999</v>
+      </c>
+      <c r="I50">
+        <v>22.128799999999998</v>
+      </c>
+      <c r="J50">
+        <v>4.6769999999999996</v>
+      </c>
+      <c r="K50">
+        <v>0.58460000000000001</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>14</v>
+      </c>
+      <c r="B51">
+        <v>2048</v>
+      </c>
+      <c r="C51">
+        <v>5</v>
+      </c>
+      <c r="D51">
+        <v>16</v>
+      </c>
+      <c r="E51">
+        <v>30</v>
+      </c>
+      <c r="F51">
+        <v>13.3993</v>
+      </c>
+      <c r="G51">
+        <v>1.3835</v>
+      </c>
+      <c r="H51">
+        <v>11.5177</v>
+      </c>
+      <c r="I51">
+        <v>17.459199999999999</v>
+      </c>
+      <c r="J51">
+        <v>6.0594000000000001</v>
+      </c>
+      <c r="K51">
+        <v>0.37869999999999998</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>14</v>
+      </c>
+      <c r="B52">
+        <v>2048</v>
+      </c>
+      <c r="C52">
+        <v>7</v>
+      </c>
+      <c r="D52">
+        <v>1</v>
+      </c>
+      <c r="E52">
+        <v>30</v>
+      </c>
+      <c r="F52">
+        <v>153.59360000000001</v>
+      </c>
+      <c r="G52">
+        <v>4.7832999999999997</v>
+      </c>
+      <c r="H52">
+        <v>150.78800000000001</v>
+      </c>
+      <c r="I52">
+        <v>177.86099999999999</v>
+      </c>
+      <c r="J52">
+        <v>1</v>
+      </c>
+      <c r="K52">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>14</v>
+      </c>
+      <c r="B53">
+        <v>2048</v>
+      </c>
+      <c r="C53">
+        <v>7</v>
+      </c>
+      <c r="D53">
+        <v>2</v>
+      </c>
+      <c r="E53">
+        <v>30</v>
+      </c>
+      <c r="F53">
+        <v>79.679900000000004</v>
+      </c>
+      <c r="G53">
+        <v>7.7319000000000004</v>
+      </c>
+      <c r="H53">
+        <v>76.503</v>
+      </c>
+      <c r="I53">
+        <v>120.117</v>
+      </c>
+      <c r="J53">
+        <v>1.9276</v>
+      </c>
+      <c r="K53">
+        <v>0.96379999999999999</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>14</v>
+      </c>
+      <c r="B54">
+        <v>2048</v>
+      </c>
+      <c r="C54">
+        <v>7</v>
+      </c>
+      <c r="D54">
+        <v>4</v>
+      </c>
+      <c r="E54">
+        <v>30</v>
+      </c>
+      <c r="F54">
+        <v>46.764600000000002</v>
+      </c>
+      <c r="G54">
+        <v>7.5646000000000004</v>
+      </c>
+      <c r="H54">
+        <v>39.732199999999999</v>
+      </c>
+      <c r="I54">
+        <v>68.224699999999999</v>
+      </c>
+      <c r="J54">
+        <v>3.2844000000000002</v>
+      </c>
+      <c r="K54">
+        <v>0.82110000000000005</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>14</v>
+      </c>
+      <c r="B55">
+        <v>2048</v>
+      </c>
+      <c r="C55">
+        <v>7</v>
+      </c>
+      <c r="D55">
+        <v>8</v>
+      </c>
+      <c r="E55">
+        <v>30</v>
+      </c>
+      <c r="F55">
+        <v>33.890999999999998</v>
+      </c>
+      <c r="G55">
+        <v>6.8665000000000003</v>
+      </c>
+      <c r="H55">
+        <v>24.648099999999999</v>
+      </c>
+      <c r="I55">
+        <v>64.464200000000005</v>
+      </c>
+      <c r="J55">
+        <v>4.532</v>
+      </c>
+      <c r="K55">
+        <v>0.5665</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>14</v>
+      </c>
+      <c r="B56">
+        <v>2048</v>
+      </c>
+      <c r="C56">
+        <v>7</v>
+      </c>
+      <c r="D56">
+        <v>16</v>
+      </c>
+      <c r="E56">
+        <v>30</v>
+      </c>
+      <c r="F56">
+        <v>28.558700000000002</v>
+      </c>
+      <c r="G56">
+        <v>2.9075000000000002</v>
+      </c>
+      <c r="H56">
+        <v>23.483499999999999</v>
+      </c>
+      <c r="I56">
+        <v>35.079900000000002</v>
+      </c>
+      <c r="J56">
+        <v>5.3781999999999996</v>
+      </c>
+      <c r="K56">
+        <v>0.33610000000000001</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>14</v>
+      </c>
+      <c r="B57">
+        <v>2048</v>
+      </c>
+      <c r="C57">
+        <v>11</v>
+      </c>
+      <c r="D57">
+        <v>1</v>
+      </c>
+      <c r="E57">
+        <v>30</v>
+      </c>
+      <c r="F57">
+        <v>406.60939999999999</v>
+      </c>
+      <c r="G57">
+        <v>4.0233999999999996</v>
+      </c>
+      <c r="H57">
+        <v>401.73700000000002</v>
+      </c>
+      <c r="I57">
+        <v>422.75099999999998</v>
+      </c>
+      <c r="J57">
+        <v>1</v>
+      </c>
+      <c r="K57">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>14</v>
+      </c>
+      <c r="B58">
+        <v>2048</v>
+      </c>
+      <c r="C58">
+        <v>11</v>
+      </c>
+      <c r="D58">
+        <v>2</v>
+      </c>
+      <c r="E58">
+        <v>30</v>
+      </c>
+      <c r="F58">
+        <v>215.00409999999999</v>
+      </c>
+      <c r="G58">
+        <v>11.483599999999999</v>
+      </c>
+      <c r="H58">
+        <v>205.34100000000001</v>
+      </c>
+      <c r="I58">
+        <v>252.72800000000001</v>
+      </c>
+      <c r="J58">
+        <v>1.8912</v>
+      </c>
+      <c r="K58">
+        <v>0.9456</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>14</v>
+      </c>
+      <c r="B59">
+        <v>2048</v>
+      </c>
+      <c r="C59">
+        <v>11</v>
+      </c>
+      <c r="D59">
+        <v>4</v>
+      </c>
+      <c r="E59">
+        <v>30</v>
+      </c>
+      <c r="F59">
+        <v>118.869</v>
+      </c>
+      <c r="G59">
+        <v>8.4090000000000007</v>
+      </c>
+      <c r="H59">
+        <v>106.462</v>
+      </c>
+      <c r="I59">
+        <v>143.06200000000001</v>
+      </c>
+      <c r="J59">
+        <v>3.4207000000000001</v>
+      </c>
+      <c r="K59">
+        <v>0.85519999999999996</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>14</v>
+      </c>
+      <c r="B60">
+        <v>2048</v>
+      </c>
+      <c r="C60">
+        <v>11</v>
+      </c>
+      <c r="D60">
+        <v>8</v>
+      </c>
+      <c r="E60">
+        <v>30</v>
+      </c>
+      <c r="F60">
+        <v>78.9268</v>
+      </c>
+      <c r="G60">
+        <v>5.4931999999999999</v>
+      </c>
+      <c r="H60">
+        <v>66.489999999999995</v>
+      </c>
+      <c r="I60">
+        <v>93.042199999999994</v>
+      </c>
+      <c r="J60">
+        <v>5.1516999999999999</v>
+      </c>
+      <c r="K60">
+        <v>0.64400000000000002</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>14</v>
+      </c>
+      <c r="B61">
+        <v>2048</v>
+      </c>
+      <c r="C61">
+        <v>11</v>
+      </c>
+      <c r="D61">
+        <v>16</v>
+      </c>
+      <c r="E61">
+        <v>30</v>
+      </c>
+      <c r="F61">
+        <v>60.029899999999998</v>
+      </c>
+      <c r="G61">
+        <v>3.3441999999999998</v>
+      </c>
+      <c r="H61">
+        <v>56.186700000000002</v>
+      </c>
+      <c r="I61">
+        <v>73.932500000000005</v>
+      </c>
+      <c r="J61">
+        <v>6.7733999999999996</v>
+      </c>
+      <c r="K61">
+        <v>0.42330000000000001</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>14</v>
+      </c>
+      <c r="B62">
+        <v>4096</v>
+      </c>
+      <c r="C62">
+        <v>3</v>
+      </c>
+      <c r="D62">
+        <v>1</v>
+      </c>
+      <c r="E62">
+        <v>30</v>
+      </c>
+      <c r="F62">
+        <v>150.49109999999999</v>
+      </c>
+      <c r="G62">
+        <v>2.8252000000000002</v>
+      </c>
+      <c r="H62">
+        <v>146.721</v>
+      </c>
+      <c r="I62">
+        <v>158.66200000000001</v>
+      </c>
+      <c r="J62">
+        <v>1</v>
+      </c>
+      <c r="K62">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>14</v>
+      </c>
+      <c r="B63">
+        <v>4096</v>
+      </c>
+      <c r="C63">
+        <v>3</v>
+      </c>
+      <c r="D63">
+        <v>2</v>
+      </c>
+      <c r="E63">
+        <v>30</v>
+      </c>
+      <c r="F63">
+        <v>77.900000000000006</v>
+      </c>
+      <c r="G63">
+        <v>3.1804999999999999</v>
+      </c>
+      <c r="H63">
+        <v>75.207499999999996</v>
+      </c>
+      <c r="I63">
+        <v>92.971500000000006</v>
+      </c>
+      <c r="J63">
+        <v>1.9318</v>
+      </c>
+      <c r="K63">
+        <v>0.96589999999999998</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>14</v>
+      </c>
+      <c r="B64">
+        <v>4096</v>
+      </c>
+      <c r="C64">
+        <v>3</v>
+      </c>
+      <c r="D64">
+        <v>4</v>
+      </c>
+      <c r="E64">
+        <v>30</v>
+      </c>
+      <c r="F64">
+        <v>49.503500000000003</v>
+      </c>
+      <c r="G64">
+        <v>7.4760999999999997</v>
+      </c>
+      <c r="H64">
+        <v>40.785299999999999</v>
+      </c>
+      <c r="I64">
+        <v>71.472800000000007</v>
+      </c>
+      <c r="J64">
+        <v>3.04</v>
+      </c>
+      <c r="K64">
+        <v>0.76</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>14</v>
+      </c>
+      <c r="B65">
+        <v>4096</v>
+      </c>
+      <c r="C65">
+        <v>3</v>
+      </c>
+      <c r="D65">
+        <v>8</v>
+      </c>
+      <c r="E65">
+        <v>30</v>
+      </c>
+      <c r="F65">
+        <v>35.290599999999998</v>
+      </c>
+      <c r="G65">
+        <v>3.6791</v>
+      </c>
+      <c r="H65">
+        <v>29.192299999999999</v>
+      </c>
+      <c r="I65">
+        <v>47.121099999999998</v>
+      </c>
+      <c r="J65">
+        <v>4.2643000000000004</v>
+      </c>
+      <c r="K65">
+        <v>0.53300000000000003</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>14</v>
+      </c>
+      <c r="B66">
+        <v>4096</v>
+      </c>
+      <c r="C66">
+        <v>3</v>
+      </c>
+      <c r="D66">
+        <v>16</v>
+      </c>
+      <c r="E66">
+        <v>30</v>
+      </c>
+      <c r="F66">
+        <v>29.472000000000001</v>
+      </c>
+      <c r="G66">
+        <v>1.9722</v>
+      </c>
+      <c r="H66">
+        <v>26.553100000000001</v>
+      </c>
+      <c r="I66">
+        <v>36.343299999999999</v>
+      </c>
+      <c r="J66">
+        <v>5.1062000000000003</v>
+      </c>
+      <c r="K66">
+        <v>0.31909999999999999</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>14</v>
+      </c>
+      <c r="B67">
+        <v>4096</v>
+      </c>
+      <c r="C67">
+        <v>5</v>
+      </c>
+      <c r="D67">
+        <v>1</v>
+      </c>
+      <c r="E67">
+        <v>30</v>
+      </c>
+      <c r="F67">
+        <v>330.6764</v>
+      </c>
+      <c r="G67">
+        <v>8.1809999999999992</v>
+      </c>
+      <c r="H67">
+        <v>325.16399999999999</v>
+      </c>
+      <c r="I67">
+        <v>363.79700000000003</v>
+      </c>
+      <c r="J67">
+        <v>1</v>
+      </c>
+      <c r="K67">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>14</v>
+      </c>
+      <c r="B68">
+        <v>4096</v>
+      </c>
+      <c r="C68">
+        <v>5</v>
+      </c>
+      <c r="D68">
+        <v>2</v>
+      </c>
+      <c r="E68">
+        <v>30</v>
+      </c>
+      <c r="F68">
+        <v>179.39500000000001</v>
+      </c>
+      <c r="G68">
+        <v>13.559100000000001</v>
+      </c>
+      <c r="H68">
+        <v>168.16399999999999</v>
+      </c>
+      <c r="I68">
+        <v>215.31200000000001</v>
+      </c>
+      <c r="J68">
+        <v>1.8432999999999999</v>
+      </c>
+      <c r="K68">
+        <v>0.92159999999999997</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
+        <v>14</v>
+      </c>
+      <c r="B69">
+        <v>4096</v>
+      </c>
+      <c r="C69">
+        <v>5</v>
+      </c>
+      <c r="D69">
+        <v>4</v>
+      </c>
+      <c r="E69">
+        <v>30</v>
+      </c>
+      <c r="F69">
+        <v>101.9585</v>
+      </c>
+      <c r="G69">
+        <v>9.0792000000000002</v>
+      </c>
+      <c r="H69">
+        <v>90.827799999999996</v>
+      </c>
+      <c r="I69">
+        <v>121.11499999999999</v>
+      </c>
+      <c r="J69">
+        <v>3.2431999999999999</v>
+      </c>
+      <c r="K69">
+        <v>0.81079999999999997</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
+        <v>14</v>
+      </c>
+      <c r="B70">
+        <v>4096</v>
+      </c>
+      <c r="C70">
+        <v>5</v>
+      </c>
+      <c r="D70">
+        <v>8</v>
+      </c>
+      <c r="E70">
+        <v>30</v>
+      </c>
+      <c r="F70">
+        <v>84.401399999999995</v>
+      </c>
+      <c r="G70">
+        <v>11.9794</v>
+      </c>
+      <c r="H70">
+        <v>63.466700000000003</v>
+      </c>
+      <c r="I70">
+        <v>114.428</v>
+      </c>
+      <c r="J70">
+        <v>3.9178999999999999</v>
+      </c>
+      <c r="K70">
+        <v>0.48970000000000002</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A71" t="s">
+        <v>14</v>
+      </c>
+      <c r="B71">
+        <v>4096</v>
+      </c>
+      <c r="C71">
+        <v>5</v>
+      </c>
+      <c r="D71">
+        <v>16</v>
+      </c>
+      <c r="E71">
+        <v>30</v>
+      </c>
+      <c r="F71">
+        <v>66.070099999999996</v>
+      </c>
+      <c r="G71">
+        <v>6.6698000000000004</v>
+      </c>
+      <c r="H71">
+        <v>56.775399999999998</v>
+      </c>
+      <c r="I71">
+        <v>82.164500000000004</v>
+      </c>
+      <c r="J71">
+        <v>5.0049000000000001</v>
+      </c>
+      <c r="K71">
+        <v>0.31280000000000002</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A72" t="s">
+        <v>14</v>
+      </c>
+      <c r="B72">
+        <v>4096</v>
+      </c>
+      <c r="C72">
+        <v>7</v>
+      </c>
+      <c r="D72">
+        <v>1</v>
+      </c>
+      <c r="E72">
+        <v>30</v>
+      </c>
+      <c r="F72">
+        <v>635.03290000000004</v>
+      </c>
+      <c r="G72">
+        <v>16.475200000000001</v>
+      </c>
+      <c r="H72">
+        <v>616.55700000000002</v>
+      </c>
+      <c r="I72">
+        <v>672.46900000000005</v>
+      </c>
+      <c r="J72">
+        <v>1</v>
+      </c>
+      <c r="K72">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A73" t="s">
+        <v>14</v>
+      </c>
+      <c r="B73">
+        <v>4096</v>
+      </c>
+      <c r="C73">
+        <v>7</v>
+      </c>
+      <c r="D73">
+        <v>2</v>
+      </c>
+      <c r="E73">
+        <v>30</v>
+      </c>
+      <c r="F73">
+        <v>330.69369999999998</v>
+      </c>
+      <c r="G73">
+        <v>20.5669</v>
+      </c>
+      <c r="H73">
+        <v>312.74299999999999</v>
+      </c>
+      <c r="I73">
+        <v>425.10700000000003</v>
+      </c>
+      <c r="J73">
+        <v>1.9202999999999999</v>
+      </c>
+      <c r="K73">
+        <v>0.96020000000000005</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A74" t="s">
+        <v>14</v>
+      </c>
+      <c r="B74">
+        <v>4096</v>
+      </c>
+      <c r="C74">
+        <v>7</v>
+      </c>
+      <c r="D74">
+        <v>4</v>
+      </c>
+      <c r="E74">
+        <v>30</v>
+      </c>
+      <c r="F74">
+        <v>194.8108</v>
+      </c>
+      <c r="G74">
+        <v>16.744800000000001</v>
+      </c>
+      <c r="H74">
+        <v>169.477</v>
+      </c>
+      <c r="I74">
+        <v>244.09299999999999</v>
+      </c>
+      <c r="J74">
+        <v>3.2597</v>
+      </c>
+      <c r="K74">
+        <v>0.81489999999999996</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A75" t="s">
+        <v>14</v>
+      </c>
+      <c r="B75">
+        <v>4096</v>
+      </c>
+      <c r="C75">
+        <v>7</v>
+      </c>
+      <c r="D75">
+        <v>8</v>
+      </c>
+      <c r="E75">
+        <v>30</v>
+      </c>
+      <c r="F75">
+        <v>131.17330000000001</v>
+      </c>
+      <c r="G75">
+        <v>12.305</v>
+      </c>
+      <c r="H75">
+        <v>115.325</v>
+      </c>
+      <c r="I75">
+        <v>178.41800000000001</v>
+      </c>
+      <c r="J75">
+        <v>4.8411999999999997</v>
+      </c>
+      <c r="K75">
+        <v>0.60509999999999997</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A76" t="s">
+        <v>14</v>
+      </c>
+      <c r="B76">
+        <v>4096</v>
+      </c>
+      <c r="C76">
+        <v>7</v>
+      </c>
+      <c r="D76">
+        <v>16</v>
+      </c>
+      <c r="E76">
+        <v>30</v>
+      </c>
+      <c r="F76">
+        <v>109.8854</v>
+      </c>
+      <c r="G76">
+        <v>10.520300000000001</v>
+      </c>
+      <c r="H76">
+        <v>97.397199999999998</v>
+      </c>
+      <c r="I76">
+        <v>151.58600000000001</v>
+      </c>
+      <c r="J76">
+        <v>5.7789999999999999</v>
+      </c>
+      <c r="K76">
+        <v>0.36120000000000002</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A77" t="s">
+        <v>14</v>
+      </c>
+      <c r="B77">
+        <v>4096</v>
+      </c>
+      <c r="C77">
+        <v>11</v>
+      </c>
+      <c r="D77">
+        <v>1</v>
+      </c>
+      <c r="E77">
+        <v>30</v>
+      </c>
+      <c r="F77">
+        <v>1629.8869999999999</v>
+      </c>
+      <c r="G77">
+        <v>19.822800000000001</v>
+      </c>
+      <c r="H77">
+        <v>1610.4</v>
+      </c>
+      <c r="I77">
+        <v>1682.71</v>
+      </c>
+      <c r="J77">
+        <v>1</v>
+      </c>
+      <c r="K77">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A78" t="s">
+        <v>14</v>
+      </c>
+      <c r="B78">
+        <v>4096</v>
+      </c>
+      <c r="C78">
+        <v>11</v>
+      </c>
+      <c r="D78">
+        <v>2</v>
+      </c>
+      <c r="E78">
+        <v>30</v>
+      </c>
+      <c r="F78">
+        <v>851.16510000000005</v>
+      </c>
+      <c r="G78">
+        <v>24.580200000000001</v>
+      </c>
+      <c r="H78">
+        <v>821.54700000000003</v>
+      </c>
+      <c r="I78">
+        <v>919.77099999999996</v>
+      </c>
+      <c r="J78">
+        <v>1.9149</v>
+      </c>
+      <c r="K78">
+        <v>0.95740000000000003</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A79" t="s">
+        <v>14</v>
+      </c>
+      <c r="B79">
+        <v>4096</v>
+      </c>
+      <c r="C79">
+        <v>11</v>
+      </c>
+      <c r="D79">
+        <v>4</v>
+      </c>
+      <c r="E79">
+        <v>30</v>
+      </c>
+      <c r="F79">
+        <v>487.21719999999999</v>
+      </c>
+      <c r="G79">
+        <v>26.899100000000001</v>
+      </c>
+      <c r="H79">
+        <v>459.30099999999999</v>
+      </c>
+      <c r="I79">
+        <v>564.23</v>
+      </c>
+      <c r="J79">
+        <v>3.3452999999999999</v>
+      </c>
+      <c r="K79">
+        <v>0.83630000000000004</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A80" t="s">
+        <v>14</v>
+      </c>
+      <c r="B80">
+        <v>4096</v>
+      </c>
+      <c r="C80">
+        <v>11</v>
+      </c>
+      <c r="D80">
+        <v>8</v>
+      </c>
+      <c r="E80">
+        <v>30</v>
+      </c>
+      <c r="F80">
+        <v>304.27429999999998</v>
+      </c>
+      <c r="G80">
+        <v>15.9878</v>
+      </c>
+      <c r="H80">
+        <v>272.524</v>
+      </c>
+      <c r="I80">
+        <v>352.048</v>
+      </c>
+      <c r="J80">
+        <v>5.3566000000000003</v>
+      </c>
+      <c r="K80">
+        <v>0.66959999999999997</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A81" t="s">
+        <v>14</v>
+      </c>
+      <c r="B81">
+        <v>4096</v>
+      </c>
+      <c r="C81">
+        <v>11</v>
+      </c>
+      <c r="D81">
+        <v>16</v>
+      </c>
+      <c r="E81">
+        <v>30</v>
+      </c>
+      <c r="F81">
+        <v>203.69489999999999</v>
+      </c>
+      <c r="G81">
+        <v>13.1831</v>
+      </c>
+      <c r="H81">
+        <v>192.27099999999999</v>
+      </c>
+      <c r="I81">
+        <v>260.86099999999999</v>
+      </c>
+      <c r="J81">
+        <v>8.0015999999999998</v>
+      </c>
+      <c r="K81">
+        <v>0.50009999999999999</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>